<commit_message>
Pin Status Anterior to baseline, remap status 8->7, add per-item status flowchart
- Status logic: Status Anterior is now pinned to a fixed baseline snapshot
  (does not shift the current status into previous on each update); Status
  Atual comes from the latest GTO (now 27/07 11:52)
- Normalize status '8 - Awaiting full B05 completion' to
  '7 - Missing Vacuum Test or Sign' everywhere (status 8 does not exist)
- Record status history per snapshot; build a per-item timeline and show it
  as a clickable flowchart modal in the dashboard (click the item number)
- Excel: new 'Item History' sheet with each item's status timeline
- Source file: tolerant to any GTO*.xlsx name in data/, auto-consolidated
  to the canonical name; replaces the newly uploaded 11:52 export
- Update CLAUDE.md to document the new rules

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UdaRc7H5wiErcmzDcK8Lt
</commit_message>
<xml_diff>
--- a/J06_Items_Analysis.xlsx
+++ b/J06_Items_Analysis.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Merged Analysis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary by Responsible" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Status Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Item History" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Merged Analysis'!$A$3:$L$221</definedName>
@@ -69,7 +70,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -113,11 +114,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
@@ -153,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -200,9 +196,6 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -239,10 +232,10 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -637,12 +630,12 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SBR4 · GTO List of Items · gerado em 27/07/2026 10:42 · 218 itens (ActualJx = J06) · 79 pendencias abertas</t>
+          <t>SBR4 · GTO List of Items · gerado em 27/07/2026 11:52 · 218 itens (ActualJx = J06) · 79 pendencias abertas</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Última atualização: 27/07/2026 10:42</t>
+          <t>Última atualização: 27/07/2026 11:52</t>
         </is>
       </c>
     </row>
@@ -4078,10 +4071,10 @@
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I59" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I59" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -4138,10 +4131,10 @@
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I60" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I60" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -4198,10 +4191,10 @@
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I61" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -4378,10 +4371,10 @@
       </c>
       <c r="H64" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I64" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I64" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -4438,10 +4431,10 @@
       </c>
       <c r="H65" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I65" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I65" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -4558,10 +4551,10 @@
       </c>
       <c r="H67" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I67" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I67" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -5038,10 +5031,10 @@
       </c>
       <c r="H75" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I75" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -5158,10 +5151,10 @@
       </c>
       <c r="H77" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I77" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -5218,10 +5211,10 @@
       </c>
       <c r="H78" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I78" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I78" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5278,10 +5271,10 @@
       </c>
       <c r="H79" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I79" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I79" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5338,10 +5331,10 @@
       </c>
       <c r="H80" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I80" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I80" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5398,10 +5391,10 @@
       </c>
       <c r="H81" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I81" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5458,10 +5451,10 @@
       </c>
       <c r="H82" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I82" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I82" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5518,10 +5511,10 @@
       </c>
       <c r="H83" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I83" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I83" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5638,10 +5631,10 @@
       </c>
       <c r="H85" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I85" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I85" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5818,10 +5811,10 @@
       </c>
       <c r="H88" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I88" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I88" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -5998,10 +5991,10 @@
       </c>
       <c r="H91" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I91" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I91" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -6538,10 +6531,10 @@
       </c>
       <c r="H100" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I100" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I100" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -6658,10 +6651,10 @@
       </c>
       <c r="H102" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I102" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I102" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -6718,10 +6711,10 @@
       </c>
       <c r="H103" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I103" s="16" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I103" s="15" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
@@ -6958,10 +6951,10 @@
       </c>
       <c r="H107" s="14" t="inlineStr">
         <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="I107" s="15" t="inlineStr">
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="I107" s="14" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
@@ -7261,7 +7254,7 @@
           <t>4 - Under Analysis To Not Blocking</t>
         </is>
       </c>
-      <c r="I112" s="17" t="inlineStr">
+      <c r="I112" s="16" t="inlineStr">
         <is>
           <t>2 - Not Blocking</t>
         </is>
@@ -7321,7 +7314,7 @@
           <t>4 - Under Analysis To Not Blocking</t>
         </is>
       </c>
-      <c r="I113" s="17" t="inlineStr">
+      <c r="I113" s="16" t="inlineStr">
         <is>
           <t>2 - Not Blocking</t>
         </is>
@@ -8305,7 +8298,7 @@
           <t>4 - Under Analysis To Not Blocking</t>
         </is>
       </c>
-      <c r="I129" s="17" t="inlineStr">
+      <c r="I129" s="16" t="inlineStr">
         <is>
           <t>2 - Not Blocking</t>
         </is>
@@ -13933,265 +13926,265 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Open Items by Responsible (excludes closed: Validated / Not Blocking)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Responsible</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Waiting/Other</t>
         </is>
       </c>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Items</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>Ship Manager</t>
         </is>
       </c>
-      <c r="B3" s="21" t="n">
+      <c r="B3" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="21" t="n">
+      <c r="D3" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>2, 494, 613, 614, 616, 620, 621, 623, 638, 646, 667, 725, 736, 779, 781, 784, 785, 809, 1027, 1030, 3098, 3100, 3103, 3279, 3280, 3293, 3306</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="B4" s="21" t="n">
+      <c r="B4" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="C4" s="21" t="n">
+      <c r="C4" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="D4" s="21" t="n">
+      <c r="D4" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>445, 618, 619, 624, 660, 661, 733, 756, 818, 1102, 1723, 1737, 1741, 1745</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>NG (Naval Group)</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>211, 560, 564, 605, 647, 648, 649, 650, 651, 652, 654, 658</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Commissioning</t>
         </is>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>409, 673, 718, 3095, 3096, 3109, 3278, 3290, 3291, 3294</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>412, 611, 622, 3281, 3282</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>GTO</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>405, 729, 782, 3113</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>SOP</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>3099, 3295</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Quality (Onboard Inspection)</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>3285, 3289</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>PCP</t>
         </is>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>3111</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Commissioning / PCP</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>3287</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Commissioning / Quality</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C13" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="22" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>3288</t>
         </is>
@@ -14211,7 +14204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14221,69 +14214,69 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Mudanças de status na última atualização (27/07/2026 10:42) — 34 item(ns)</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Mudanças de status (Anterior → Atual) — 22 item(ns)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Status Anterior</t>
         </is>
       </c>
-      <c r="C2" s="19" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Status Atual</t>
         </is>
       </c>
-      <c r="D2" s="19" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="n">
+      <c r="A3" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C3" s="24" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>4 - Under Analysis</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>Broadcasting safety alarms to all rooms of the ship.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="n">
+      <c r="A4" s="20" t="n">
         <v>426</v>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>1 - Validated by ICN</t>
-        </is>
-      </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure.
 Entire EM circuit</t>
@@ -14291,20 +14284,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="20" t="n">
         <v>445</v>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>3 - Blocking</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>4 - Under Analysis</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure.
 Leak test of the draining circuit of tube</t>
@@ -14312,621 +14305,381 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="n">
-        <v>613</v>
-      </c>
-      <c r="B6" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="A6" s="20" t="n">
+        <v>647</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30030</t>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32004</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
-        <v>614</v>
-      </c>
-      <c r="B7" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="A7" s="20" t="n">
+        <v>648</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30040</t>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32005</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="n">
-        <v>616</v>
-      </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="A8" s="20" t="n">
+        <v>649</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30051</t>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32006</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="n">
-        <v>620</v>
-      </c>
-      <c r="B9" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="A9" s="20" t="n">
+        <v>650</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30070</t>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32007</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="n">
-        <v>621</v>
-      </c>
-      <c r="B10" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="A10" s="20" t="n">
+        <v>651</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30071</t>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32008</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="n">
-        <v>623</v>
-      </c>
-      <c r="B11" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="A11" s="20" t="n">
+        <v>652</v>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC30090</t>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32009</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="n">
-        <v>638</v>
-      </c>
-      <c r="B12" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr">
+      <c r="A12" s="20" t="n">
+        <v>654</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC31016</t>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32011</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="n">
-        <v>646</v>
-      </c>
-      <c r="B13" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="A13" s="20" t="n">
+        <v>658</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>7 - Missing Vacuum Test or Sign</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32003 - Diesel supply EQ00411 (água)</t>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>6 - Waiting B05</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32015</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="n">
-        <v>647</v>
-      </c>
-      <c r="B14" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="A14" s="20" t="n">
+        <v>729</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>6 - Waiting B05</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32004</t>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC33043</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="n">
-        <v>648</v>
-      </c>
-      <c r="B15" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D15" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32005</t>
+      <c r="A15" s="20" t="n">
+        <v>764</v>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC34040</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="n">
-        <v>649</v>
-      </c>
-      <c r="B16" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D16" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32006</t>
+      <c r="A16" s="20" t="n">
+        <v>765</v>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC34041</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="n">
-        <v>650</v>
-      </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D17" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32007</t>
+      <c r="A17" s="20" t="n">
+        <v>785</v>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Document to be produce by ICN in conformity with SOI, This includes specifically SOD_M2_CH_1-14 “Refloating”</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="n">
-        <v>651</v>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D18" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32008</t>
+      <c r="A18" s="20" t="n">
+        <v>809</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Functional test of the voice-activated telephone network</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="n">
-        <v>652</v>
-      </c>
-      <c r="B19" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32009</t>
+      <c r="A19" s="20" t="n">
+        <v>855</v>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Air renewal ventilation system: Setting Configurations</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="n">
-        <v>654</v>
-      </c>
-      <c r="B20" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32011</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="21" t="n">
-        <v>658</v>
-      </c>
-      <c r="B21" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32015</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="21" t="n">
-        <v>667</v>
-      </c>
-      <c r="B22" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C22" s="28" t="inlineStr">
-        <is>
-          <t>7 - Missing Vacuum Test or Sign</t>
-        </is>
-      </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC32030</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="21" t="n">
-        <v>718</v>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="inlineStr">
-        <is>
-          <t>7 - Missing Vacuum Test or Sign</t>
-        </is>
-      </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC33018</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="21" t="n">
-        <v>725</v>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>7 - Missing Vacuum Test or Sign</t>
-        </is>
-      </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC33028</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="21" t="n">
-        <v>729</v>
-      </c>
-      <c r="B25" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>6 - Waiting B05</t>
-        </is>
-      </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC33043</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="n">
-        <v>736</v>
-      </c>
-      <c r="B26" s="27" t="inlineStr">
-        <is>
-          <t>8 - Awaiting full B05 completion</t>
-        </is>
-      </c>
-      <c r="C26" s="28" t="inlineStr">
-        <is>
-          <t>7 - Missing Vacuum Test or Sign</t>
-        </is>
-      </c>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC33056</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="n">
-        <v>764</v>
-      </c>
-      <c r="B27" s="24" t="inlineStr">
-        <is>
-          <t>4 - Under Analysis To Not Blocking</t>
-        </is>
-      </c>
-      <c r="C27" s="30" t="inlineStr">
-        <is>
-          <t>2 - Not Blocking</t>
-        </is>
-      </c>
-      <c r="D27" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC34040</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="n">
-        <v>765</v>
-      </c>
-      <c r="B28" s="24" t="inlineStr">
-        <is>
-          <t>4 - Under Analysis To Not Blocking</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr">
-        <is>
-          <t>2 - Not Blocking</t>
-        </is>
-      </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Penetration outfitting according to “Pressure Hull integrity” plan AC34041</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="21" t="n">
-        <v>785</v>
-      </c>
-      <c r="B29" s="23" t="inlineStr">
-        <is>
-          <t>5 - Waiting Proof</t>
-        </is>
-      </c>
-      <c r="C29" s="24" t="inlineStr">
+      <c r="A20" s="20" t="n">
+        <v>1741</v>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>3 - Blocking</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>4 - Under Analysis</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
-        <is>
-          <t>Document to be produce by ICN in conformity with SOI, This includes specifically SOD_M2_CH_1-14 “Refloating”</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="n">
-        <v>809</v>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>5 - Waiting Proof</t>
-        </is>
-      </c>
-      <c r="C30" s="24" t="inlineStr">
-        <is>
-          <t>4 - Under Analysis</t>
-        </is>
-      </c>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>Functional test of the voice-activated telephone network</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="n">
-        <v>855</v>
-      </c>
-      <c r="B31" s="24" t="inlineStr">
-        <is>
-          <t>4 - Under Analysis To Not Blocking</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr">
-        <is>
-          <t>2 - Not Blocking</t>
-        </is>
-      </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Air renewal ventilation system: Setting Configurations</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="21" t="n">
-        <v>1741</v>
-      </c>
-      <c r="B32" s="26" t="inlineStr">
-        <is>
-          <t>3 - Blocking</t>
-        </is>
-      </c>
-      <c r="C32" s="24" t="inlineStr">
-        <is>
-          <t>4 - Under Analysis</t>
-        </is>
-      </c>
-      <c r="D32" s="22" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure.
 Leak test of the blowing air circuits</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="21" t="n">
+    <row r="21">
+      <c r="A21" s="20" t="n">
         <v>1761</v>
       </c>
-      <c r="B33" s="23" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>1 - Validated by ICN</t>
-        </is>
-      </c>
-      <c r="D33" s="22" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure. Leak test of compress gas circuit of MultiCom Mast</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="21" t="n">
+    <row r="22">
+      <c r="A22" s="20" t="n">
         <v>1762</v>
       </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>1 - Validated by ICN</t>
-        </is>
-      </c>
-      <c r="D34" s="22" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure. Leak test of compress gas circuit of ESM Mast</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="21" t="n">
+    <row r="23">
+      <c r="A23" s="20" t="n">
         <v>1763</v>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>1 - Validated by ICN</t>
-        </is>
-      </c>
-      <c r="D35" s="22" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Circuits subjected to submergence pressure. Leak test of compress gas circuit of Radar Mast</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="21" t="n">
+    <row r="24">
+      <c r="A24" s="20" t="n">
         <v>3287</v>
       </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>5 - Waiting Proof</t>
         </is>
       </c>
-      <c r="C36" s="24" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>4 - Under Analysis</t>
         </is>
       </c>
-      <c r="D36" s="22" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>EZ - Breathing equipment (air breathing masks with portable bottle) for teams inside the ship out of lhe firefighter equipment to be evaluated.</t>
         </is>
@@ -14938,4 +14691,2224 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B220"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Histórico de status por item (Inicial → ... → Atual)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Linha do tempo de status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="n">
+        <v>49</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="n">
+        <v>133</v>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="n">
+        <v>207</v>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="n">
+        <v>208</v>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="n">
+        <v>209</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="n">
+        <v>211</v>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="n">
+        <v>214</v>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="n">
+        <v>243</v>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="n">
+        <v>326</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="n">
+        <v>405</v>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="n">
+        <v>406</v>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="n">
+        <v>407</v>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="n">
+        <v>408</v>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="n">
+        <v>409</v>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="n">
+        <v>411</v>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="n">
+        <v>412</v>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="n">
+        <v>415</v>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="n">
+        <v>416</v>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="n">
+        <v>417</v>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="n">
+        <v>426</v>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  1 - Validated by ICN (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="n">
+        <v>432</v>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="n">
+        <v>434</v>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="n">
+        <v>435</v>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="n">
+        <v>436</v>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="n">
+        <v>437</v>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="n">
+        <v>438</v>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="n">
+        <v>439</v>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="n">
+        <v>442</v>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="n">
+        <v>443</v>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="n">
+        <v>445</v>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="n">
+        <v>446</v>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="n">
+        <v>447</v>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="n">
+        <v>451</v>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="n">
+        <v>461</v>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="n">
+        <v>462</v>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="n">
+        <v>463</v>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="n">
+        <v>487</v>
+      </c>
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="n">
+        <v>494</v>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="n">
+        <v>526</v>
+      </c>
+      <c r="B43" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="n">
+        <v>528</v>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="29" t="n">
+        <v>560</v>
+      </c>
+      <c r="B45" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="n">
+        <v>564</v>
+      </c>
+      <c r="B46" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="29" t="n">
+        <v>566</v>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="29" t="n">
+        <v>570</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="29" t="n">
+        <v>571</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="29" t="n">
+        <v>575</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="n">
+        <v>585</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="n">
+        <v>605</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="n">
+        <v>607</v>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="n">
+        <v>609</v>
+      </c>
+      <c r="B54" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="29" t="n">
+        <v>610</v>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="29" t="n">
+        <v>611</v>
+      </c>
+      <c r="B56" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="29" t="n">
+        <v>612</v>
+      </c>
+      <c r="B57" s="21" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="29" t="n">
+        <v>613</v>
+      </c>
+      <c r="B58" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="29" t="n">
+        <v>614</v>
+      </c>
+      <c r="B59" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="29" t="n">
+        <v>616</v>
+      </c>
+      <c r="B60" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="29" t="n">
+        <v>618</v>
+      </c>
+      <c r="B61" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="29" t="n">
+        <v>619</v>
+      </c>
+      <c r="B62" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="29" t="n">
+        <v>620</v>
+      </c>
+      <c r="B63" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="29" t="n">
+        <v>621</v>
+      </c>
+      <c r="B64" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="29" t="n">
+        <v>622</v>
+      </c>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="29" t="n">
+        <v>623</v>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="29" t="n">
+        <v>624</v>
+      </c>
+      <c r="B67" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="29" t="n">
+        <v>625</v>
+      </c>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="29" t="n">
+        <v>626</v>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="29" t="n">
+        <v>627</v>
+      </c>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="29" t="n">
+        <v>628</v>
+      </c>
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="29" t="n">
+        <v>629</v>
+      </c>
+      <c r="B72" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="29" t="n">
+        <v>636</v>
+      </c>
+      <c r="B73" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="29" t="n">
+        <v>638</v>
+      </c>
+      <c r="B74" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="29" t="n">
+        <v>645</v>
+      </c>
+      <c r="B75" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="29" t="n">
+        <v>646</v>
+      </c>
+      <c r="B76" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="29" t="n">
+        <v>647</v>
+      </c>
+      <c r="B77" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="29" t="n">
+        <v>648</v>
+      </c>
+      <c r="B78" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="29" t="n">
+        <v>649</v>
+      </c>
+      <c r="B79" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="29" t="n">
+        <v>650</v>
+      </c>
+      <c r="B80" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="29" t="n">
+        <v>651</v>
+      </c>
+      <c r="B81" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="29" t="n">
+        <v>652</v>
+      </c>
+      <c r="B82" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="29" t="n">
+        <v>653</v>
+      </c>
+      <c r="B83" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="29" t="n">
+        <v>654</v>
+      </c>
+      <c r="B84" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="29" t="n">
+        <v>655</v>
+      </c>
+      <c r="B85" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="29" t="n">
+        <v>657</v>
+      </c>
+      <c r="B86" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="29" t="n">
+        <v>658</v>
+      </c>
+      <c r="B87" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="29" t="n">
+        <v>660</v>
+      </c>
+      <c r="B88" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="29" t="n">
+        <v>661</v>
+      </c>
+      <c r="B89" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="29" t="n">
+        <v>667</v>
+      </c>
+      <c r="B90" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="29" t="n">
+        <v>673</v>
+      </c>
+      <c r="B91" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="29" t="n">
+        <v>676</v>
+      </c>
+      <c r="B92" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="n">
+        <v>704</v>
+      </c>
+      <c r="B93" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="29" t="n">
+        <v>705</v>
+      </c>
+      <c r="B94" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="29" t="n">
+        <v>706</v>
+      </c>
+      <c r="B95" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="29" t="n">
+        <v>708</v>
+      </c>
+      <c r="B96" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="29" t="n">
+        <v>711</v>
+      </c>
+      <c r="B97" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="29" t="n">
+        <v>714</v>
+      </c>
+      <c r="B98" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="29" t="n">
+        <v>718</v>
+      </c>
+      <c r="B99" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="29" t="n">
+        <v>719</v>
+      </c>
+      <c r="B100" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="29" t="n">
+        <v>725</v>
+      </c>
+      <c r="B101" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="29" t="n">
+        <v>729</v>
+      </c>
+      <c r="B102" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)  →  6 - Waiting B05 (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="29" t="n">
+        <v>730</v>
+      </c>
+      <c r="B103" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="29" t="n">
+        <v>732</v>
+      </c>
+      <c r="B104" s="21" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="29" t="n">
+        <v>733</v>
+      </c>
+      <c r="B105" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="29" t="n">
+        <v>736</v>
+      </c>
+      <c r="B106" s="21" t="inlineStr">
+        <is>
+          <t>7 - Missing Vacuum Test or Sign (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="29" t="n">
+        <v>743</v>
+      </c>
+      <c r="B107" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="29" t="n">
+        <v>751</v>
+      </c>
+      <c r="B108" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="29" t="n">
+        <v>752</v>
+      </c>
+      <c r="B109" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="29" t="n">
+        <v>756</v>
+      </c>
+      <c r="B110" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="29" t="n">
+        <v>764</v>
+      </c>
+      <c r="B111" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking (Inicial)  →  2 - Not Blocking (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="29" t="n">
+        <v>765</v>
+      </c>
+      <c r="B112" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking (Inicial)  →  2 - Not Blocking (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="29" t="n">
+        <v>777</v>
+      </c>
+      <c r="B113" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="29" t="n">
+        <v>779</v>
+      </c>
+      <c r="B114" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="29" t="n">
+        <v>780</v>
+      </c>
+      <c r="B115" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="29" t="n">
+        <v>781</v>
+      </c>
+      <c r="B116" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="29" t="n">
+        <v>782</v>
+      </c>
+      <c r="B117" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="29" t="n">
+        <v>783</v>
+      </c>
+      <c r="B118" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="29" t="n">
+        <v>784</v>
+      </c>
+      <c r="B119" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="29" t="n">
+        <v>785</v>
+      </c>
+      <c r="B120" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="29" t="n">
+        <v>786</v>
+      </c>
+      <c r="B121" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="29" t="n">
+        <v>809</v>
+      </c>
+      <c r="B122" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="29" t="n">
+        <v>817</v>
+      </c>
+      <c r="B123" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="29" t="n">
+        <v>818</v>
+      </c>
+      <c r="B124" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="29" t="n">
+        <v>820</v>
+      </c>
+      <c r="B125" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="29" t="n">
+        <v>822</v>
+      </c>
+      <c r="B126" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="29" t="n">
+        <v>840</v>
+      </c>
+      <c r="B127" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="29" t="n">
+        <v>855</v>
+      </c>
+      <c r="B128" s="21" t="inlineStr">
+        <is>
+          <t>4 - Under Analysis To Not Blocking (Inicial)  →  2 - Not Blocking (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="29" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B129" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="29" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B130" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="29" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B131" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="29" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B132" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="29" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B133" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="29" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B134" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="29" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B135" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="29" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B136" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="29" t="n">
+        <v>1025</v>
+      </c>
+      <c r="B137" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="29" t="n">
+        <v>1026</v>
+      </c>
+      <c r="B138" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="29" t="n">
+        <v>1027</v>
+      </c>
+      <c r="B139" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="29" t="n">
+        <v>1029</v>
+      </c>
+      <c r="B140" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="29" t="n">
+        <v>1030</v>
+      </c>
+      <c r="B141" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="29" t="n">
+        <v>1102</v>
+      </c>
+      <c r="B142" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="29" t="n">
+        <v>1110</v>
+      </c>
+      <c r="B143" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="29" t="n">
+        <v>1193</v>
+      </c>
+      <c r="B144" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="29" t="n">
+        <v>1576</v>
+      </c>
+      <c r="B145" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="29" t="n">
+        <v>1618</v>
+      </c>
+      <c r="B146" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="29" t="n">
+        <v>1619</v>
+      </c>
+      <c r="B147" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="29" t="n">
+        <v>1620</v>
+      </c>
+      <c r="B148" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="29" t="n">
+        <v>1621</v>
+      </c>
+      <c r="B149" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="29" t="n">
+        <v>1723</v>
+      </c>
+      <c r="B150" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="29" t="n">
+        <v>1724</v>
+      </c>
+      <c r="B151" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="29" t="n">
+        <v>1726</v>
+      </c>
+      <c r="B152" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="29" t="n">
+        <v>1731</v>
+      </c>
+      <c r="B153" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="29" t="n">
+        <v>1732</v>
+      </c>
+      <c r="B154" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="29" t="n">
+        <v>1733</v>
+      </c>
+      <c r="B155" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="29" t="n">
+        <v>1734</v>
+      </c>
+      <c r="B156" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="29" t="n">
+        <v>1735</v>
+      </c>
+      <c r="B157" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="29" t="n">
+        <v>1736</v>
+      </c>
+      <c r="B158" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="29" t="n">
+        <v>1737</v>
+      </c>
+      <c r="B159" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="29" t="n">
+        <v>1738</v>
+      </c>
+      <c r="B160" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="29" t="n">
+        <v>1739</v>
+      </c>
+      <c r="B161" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="29" t="n">
+        <v>1740</v>
+      </c>
+      <c r="B162" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="29" t="n">
+        <v>1741</v>
+      </c>
+      <c r="B163" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="29" t="n">
+        <v>1744</v>
+      </c>
+      <c r="B164" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="29" t="n">
+        <v>1745</v>
+      </c>
+      <c r="B165" s="21" t="inlineStr">
+        <is>
+          <t>3 - Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="29" t="n">
+        <v>1746</v>
+      </c>
+      <c r="B166" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="29" t="n">
+        <v>1747</v>
+      </c>
+      <c r="B167" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="29" t="n">
+        <v>1748</v>
+      </c>
+      <c r="B168" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="29" t="n">
+        <v>1749</v>
+      </c>
+      <c r="B169" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="29" t="n">
+        <v>1750</v>
+      </c>
+      <c r="B170" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="29" t="n">
+        <v>1751</v>
+      </c>
+      <c r="B171" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="29" t="n">
+        <v>1752</v>
+      </c>
+      <c r="B172" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="29" t="n">
+        <v>1753</v>
+      </c>
+      <c r="B173" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="29" t="n">
+        <v>1754</v>
+      </c>
+      <c r="B174" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="29" t="n">
+        <v>1755</v>
+      </c>
+      <c r="B175" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="29" t="n">
+        <v>1758</v>
+      </c>
+      <c r="B176" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="29" t="n">
+        <v>1759</v>
+      </c>
+      <c r="B177" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="29" t="n">
+        <v>1760</v>
+      </c>
+      <c r="B178" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="29" t="n">
+        <v>1761</v>
+      </c>
+      <c r="B179" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  1 - Validated by ICN (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="29" t="n">
+        <v>1762</v>
+      </c>
+      <c r="B180" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  1 - Validated by ICN (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="29" t="n">
+        <v>1763</v>
+      </c>
+      <c r="B181" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  1 - Validated by ICN (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="29" t="n">
+        <v>1764</v>
+      </c>
+      <c r="B182" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="29" t="n">
+        <v>1765</v>
+      </c>
+      <c r="B183" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="29" t="n">
+        <v>3005</v>
+      </c>
+      <c r="B184" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="29" t="n">
+        <v>3095</v>
+      </c>
+      <c r="B185" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="29" t="n">
+        <v>3096</v>
+      </c>
+      <c r="B186" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="29" t="n">
+        <v>3097</v>
+      </c>
+      <c r="B187" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="29" t="n">
+        <v>3098</v>
+      </c>
+      <c r="B188" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="29" t="n">
+        <v>3099</v>
+      </c>
+      <c r="B189" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="29" t="n">
+        <v>3100</v>
+      </c>
+      <c r="B190" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="29" t="n">
+        <v>3101</v>
+      </c>
+      <c r="B191" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="29" t="n">
+        <v>3102</v>
+      </c>
+      <c r="B192" s="21" t="inlineStr">
+        <is>
+          <t>2 - Not Blocking (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="29" t="n">
+        <v>3103</v>
+      </c>
+      <c r="B193" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="29" t="n">
+        <v>3105</v>
+      </c>
+      <c r="B194" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="29" t="n">
+        <v>3106</v>
+      </c>
+      <c r="B195" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="29" t="n">
+        <v>3107</v>
+      </c>
+      <c r="B196" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="29" t="n">
+        <v>3109</v>
+      </c>
+      <c r="B197" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="29" t="n">
+        <v>3111</v>
+      </c>
+      <c r="B198" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="29" t="n">
+        <v>3113</v>
+      </c>
+      <c r="B199" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="29" t="n">
+        <v>3277</v>
+      </c>
+      <c r="B200" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="29" t="n">
+        <v>3278</v>
+      </c>
+      <c r="B201" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="29" t="n">
+        <v>3279</v>
+      </c>
+      <c r="B202" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="29" t="n">
+        <v>3280</v>
+      </c>
+      <c r="B203" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="29" t="n">
+        <v>3281</v>
+      </c>
+      <c r="B204" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="29" t="n">
+        <v>3282</v>
+      </c>
+      <c r="B205" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="29" t="n">
+        <v>3284</v>
+      </c>
+      <c r="B206" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="29" t="n">
+        <v>3285</v>
+      </c>
+      <c r="B207" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="29" t="n">
+        <v>3286</v>
+      </c>
+      <c r="B208" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="29" t="n">
+        <v>3287</v>
+      </c>
+      <c r="B209" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)  →  4 - Under Analysis (27/07 10:42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="29" t="n">
+        <v>3288</v>
+      </c>
+      <c r="B210" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="29" t="n">
+        <v>3289</v>
+      </c>
+      <c r="B211" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="29" t="n">
+        <v>3290</v>
+      </c>
+      <c r="B212" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="29" t="n">
+        <v>3291</v>
+      </c>
+      <c r="B213" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="29" t="n">
+        <v>3292</v>
+      </c>
+      <c r="B214" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="29" t="n">
+        <v>3293</v>
+      </c>
+      <c r="B215" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="29" t="n">
+        <v>3294</v>
+      </c>
+      <c r="B216" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="29" t="n">
+        <v>3295</v>
+      </c>
+      <c r="B217" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="29" t="n">
+        <v>3298</v>
+      </c>
+      <c r="B218" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="29" t="n">
+        <v>3299</v>
+      </c>
+      <c r="B219" s="21" t="inlineStr">
+        <is>
+          <t>1 - Validated by ICN (Inicial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="29" t="n">
+        <v>3306</v>
+      </c>
+      <c r="B220" s="21" t="inlineStr">
+        <is>
+          <t>5 - Waiting Proof (Inicial)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update item responsibles from uploaded J06_Items_Analysis_002.xlsx
- Sync the Responsible of every item from the user-provided file into
  data/enrichment.json (source of curated responsibles)
- Net effect: 7 real reassignments (622, 624, 676, 1027, 1030, 3285, 3288);
  the closed-item placeholder is recomputed by the build
- Regenerate dashboard and Excel; responsibles now match the file exactly
</commit_message>
<xml_diff>
--- a/J06_Items_Analysis.xlsx
+++ b/J06_Items_Analysis.xlsx
@@ -4506,7 +4506,7 @@
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Quality</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Quality</t>
+          <t>NG (Naval Group)</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr">
@@ -6120,7 +6120,11 @@
         </is>
       </c>
       <c r="J93" s="6" t="inlineStr"/>
-      <c r="K93" s="6" t="inlineStr"/>
+      <c r="K93" s="6" t="inlineStr">
+        <is>
+          <t>Commissioning</t>
+        </is>
+      </c>
       <c r="L93" s="6" t="inlineStr"/>
     </row>
     <row r="94">
@@ -8965,7 +8969,7 @@
       </c>
       <c r="K140" s="6" t="inlineStr">
         <is>
-          <t>Ship Manager</t>
+          <t>Commissioning</t>
         </is>
       </c>
       <c r="L140" s="6" t="inlineStr">
@@ -9085,7 +9089,7 @@
       </c>
       <c r="K142" s="6" t="inlineStr">
         <is>
-          <t>Ship Manager</t>
+          <t>Commissioning</t>
         </is>
       </c>
       <c r="L142" s="6" t="inlineStr">
@@ -13094,7 +13098,7 @@
       </c>
       <c r="K208" s="6" t="inlineStr">
         <is>
-          <t>Quality (Onboard Inspection)</t>
+          <t>Ship Manager</t>
         </is>
       </c>
       <c r="L208" s="6" t="inlineStr">
@@ -13274,7 +13278,7 @@
       </c>
       <c r="K211" s="6" t="inlineStr">
         <is>
-          <t>Commissioning / Quality</t>
+          <t>Commissioning</t>
         </is>
       </c>
       <c r="L211" s="6" t="inlineStr">
@@ -13903,7 +13907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13954,17 +13958,17 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="20" t="n">
         <v>21</v>
       </c>
       <c r="E3" s="21" t="inlineStr">
         <is>
-          <t>2, 613, 614, 616, 620, 621, 623, 638, 646, 667, 725, 736, 784, 1027, 1030, 3098, 3100, 3103, 3279, 3280, 3293, 3306</t>
+          <t>2, 613, 614, 616, 620, 621, 623, 638, 646, 667, 725, 736, 784, 3098, 3100, 3103, 3279, 3280, 3285, 3293, 3306</t>
         </is>
       </c>
     </row>
@@ -13975,17 +13979,17 @@
         </is>
       </c>
       <c r="B4" s="20" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="20" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>409, 673, 718, 3095, 3096, 3109, 3278, 3290, 3291, 3294</t>
+          <t>409, 673, 676, 718, 1027, 1030, 3095, 3096, 3109, 3278, 3288, 3290, 3291, 3294</t>
         </is>
       </c>
     </row>
@@ -14006,35 +14010,35 @@
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>618, 619, 624, 660, 661, 733, 756, 1102, 1745</t>
+          <t>618, 619, 622, 660, 661, 733, 756, 1102, 1745</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>NG (Naval Group)</t>
         </is>
       </c>
       <c r="B6" s="20" t="n">
         <v>4</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>611, 622, 3281, 3282</t>
+          <t>211, 560, 564, 624</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>NG (Naval Group)</t>
+          <t>GTO</t>
         </is>
       </c>
       <c r="B7" s="20" t="n">
@@ -14048,28 +14052,28 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>211, 560, 564</t>
+          <t>405, 782, 3113</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>GTO</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>405, 782, 3113</t>
+          <t>611, 3281, 3282</t>
         </is>
       </c>
     </row>
@@ -14097,49 +14101,49 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>Quality (Onboard Inspection)</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="20" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>3285, 3289</t>
+          <t>3111</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>(To be assigned)</t>
+          <t>Commissioning / PCP</t>
         </is>
       </c>
       <c r="B11" s="20" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="20" t="n">
-        <v>0</v>
-      </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>676</t>
+          <t>3287</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Quality (Onboard Inspection)</t>
         </is>
       </c>
       <c r="B12" s="20" t="n">
@@ -14153,49 +14157,7 @@
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>3111</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>Commissioning / PCP</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>3287</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>Commissioning / Quality</t>
-        </is>
-      </c>
-      <c r="B14" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="21" t="inlineStr">
-        <is>
-          <t>3288</t>
+          <t>3289</t>
         </is>
       </c>
     </row>

</xml_diff>